<commit_message>
Added code that fixes not adding cities become infected
</commit_message>
<xml_diff>
--- a/Camping_data/Parks_and_camping_Master_2022-02-24.xlsx
+++ b/Camping_data/Parks_and_camping_Master_2022-02-24.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25225"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unbcloud-my.sharepoint.com/personal/acaouett_unb_ca/Documents/Grad Studies/EAB_Model/Coding/Camping_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="8_{4DEA18F6-B857-42BC-A09E-3D0FF45B6CBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FC6C3493-EF2D-45E4-9C25-834AD8496691}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="8_{4DEA18F6-B857-42BC-A09E-3D0FF45B6CBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4A7B114-C905-461D-9350-28FE7B1FEE69}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{3711D111-1412-4D58-BE4C-87E6B68A2B9C}"/>
   </bookViews>
@@ -5530,15 +5530,15 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -5546,70 +5546,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="8">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Verdana"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Verdana"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Verdana"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.00000000"/>
       <fill>
@@ -5645,6 +5581,70 @@
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Verdana"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Verdana"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Verdana"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -5728,20 +5728,26 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D6CD4C8E-0FED-4C68-89EF-51355D49EE58}" name="Table2" displayName="Table2" ref="A1:O229" totalsRowShown="0">
-  <autoFilter ref="A1:O229" xr:uid="{C0C332D5-F1AF-4545-A240-5D3F857235FD}"/>
+  <autoFilter ref="A1:O229" xr:uid="{C0C332D5-F1AF-4545-A240-5D3F857235FD}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="PE"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:O229">
     <sortCondition ref="C1:C229"/>
   </sortState>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{112FB325-F4BD-4744-9AA4-3D3AB6B90E18}" name="Type of Campground" dataDxfId="2"/>
-    <tableColumn id="17" xr3:uid="{F918C5DF-0904-479B-A7C2-45E20628DDE7}" name="Key" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{128BA3DE-B292-468A-948A-F877B5AC4312}" name="Name" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{112FB325-F4BD-4744-9AA4-3D3AB6B90E18}" name="Type of Campground" dataDxfId="7"/>
+    <tableColumn id="17" xr3:uid="{F918C5DF-0904-479B-A7C2-45E20628DDE7}" name="Key" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{128BA3DE-B292-468A-948A-F877B5AC4312}" name="Name" dataDxfId="5"/>
     <tableColumn id="3" xr3:uid="{F1734D31-AEAA-4E19-9694-721E4FD655AB}" name="Province"/>
-    <tableColumn id="4" xr3:uid="{5FF2BCCD-52F9-496E-8EDF-D1D7E45C9B6E}" name="Sites" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{7471EC6B-A3C5-4C16-8F1C-A00B00F6974B}" name="Nightly" dataDxfId="6"/>
-    <tableColumn id="13" xr3:uid="{DCE062C9-2E4C-4769-A20B-1C1ECF79BEA8}" name="Seasonal" dataDxfId="5"/>
-    <tableColumn id="10" xr3:uid="{2B490CF2-1F9E-4CFB-A004-138A307511CD}" name="Latitude" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{B0E127EB-7799-43D7-8956-C74679607620}" name="Longitude" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{5FF2BCCD-52F9-496E-8EDF-D1D7E45C9B6E}" name="Sites" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{7471EC6B-A3C5-4C16-8F1C-A00B00F6974B}" name="Nightly" dataDxfId="3"/>
+    <tableColumn id="13" xr3:uid="{DCE062C9-2E4C-4769-A20B-1C1ECF79BEA8}" name="Seasonal" dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{2B490CF2-1F9E-4CFB-A004-138A307511CD}" name="Latitude" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{B0E127EB-7799-43D7-8956-C74679607620}" name="Longitude" dataDxfId="0"/>
     <tableColumn id="9" xr3:uid="{82A7D426-6D2C-459C-B342-F7D78316E616}" name="Aquiring firewood"/>
     <tableColumn id="5" xr3:uid="{4E8695E9-2FD8-4934-9BB4-A0D492D9ED35}" name="Notes"/>
     <tableColumn id="8" xr3:uid="{FC0DEABF-2F23-4BAB-87F9-0D1D70F1AE81}" name="Phone Number"/>
@@ -6371,7 +6377,7 @@
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="19.36328125" customWidth="1"/>
-    <col min="2" max="3" width="25.453125" style="86" customWidth="1"/>
+    <col min="2" max="3" width="25.453125" style="84" customWidth="1"/>
     <col min="4" max="5" width="25.453125" customWidth="1"/>
     <col min="6" max="6" width="18.81640625" customWidth="1"/>
     <col min="7" max="7" width="11.453125" customWidth="1"/>
@@ -6393,7 +6399,7 @@
       <c r="A1" t="s">
         <v>1402</v>
       </c>
-      <c r="B1" s="86" t="s">
+      <c r="B1" s="84" t="s">
         <v>1638</v>
       </c>
       <c r="C1" t="s">
@@ -6445,11 +6451,11 @@
         <v>1244</v>
       </c>
     </row>
-    <row r="2" spans="1:21" ht="27">
+    <row r="2" spans="1:21" ht="27" hidden="1">
       <c r="A2" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="87" t="s">
+      <c r="B2" s="85" t="s">
         <v>1410</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -6490,11 +6496,11 @@
       </c>
       <c r="Q2" s="71"/>
     </row>
-    <row r="3" spans="1:21" ht="40.5">
+    <row r="3" spans="1:21" ht="40.5" hidden="1">
       <c r="A3" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B3" s="87" t="s">
+      <c r="B3" s="85" t="s">
         <v>1411</v>
       </c>
       <c r="C3" s="3" t="s">
@@ -6546,11 +6552,11 @@
         <v>1233</v>
       </c>
     </row>
-    <row r="4" spans="1:21">
+    <row r="4" spans="1:21" hidden="1">
       <c r="A4" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B4" s="87" t="s">
+      <c r="B4" s="85" t="s">
         <v>1412</v>
       </c>
       <c r="C4" s="3" t="s">
@@ -6606,7 +6612,7 @@
       <c r="A5" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B5" s="87" t="s">
+      <c r="B5" s="85" t="s">
         <v>1413</v>
       </c>
       <c r="C5" s="3" t="s">
@@ -6658,11 +6664,11 @@
         <v>1265</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="27">
+    <row r="6" spans="1:21" ht="27" hidden="1">
       <c r="A6" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B6" s="87" t="s">
+      <c r="B6" s="85" t="s">
         <v>1414</v>
       </c>
       <c r="C6" s="3" t="s">
@@ -6704,11 +6710,11 @@
         <v>1360</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="27" customHeight="1">
+    <row r="7" spans="1:21" ht="27" hidden="1" customHeight="1">
       <c r="A7" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B7" s="87" t="s">
+      <c r="B7" s="85" t="s">
         <v>1415</v>
       </c>
       <c r="C7" s="3" t="s">
@@ -6762,11 +6768,11 @@
       <c r="T7" s="4"/>
       <c r="U7" s="5"/>
     </row>
-    <row r="8" spans="1:21" ht="27">
+    <row r="8" spans="1:21" ht="27" hidden="1">
       <c r="A8" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="87" t="s">
+      <c r="B8" s="85" t="s">
         <v>1416</v>
       </c>
       <c r="C8" s="3" t="s">
@@ -6809,11 +6815,11 @@
         <v>1397</v>
       </c>
     </row>
-    <row r="9" spans="1:21" ht="27" customHeight="1">
+    <row r="9" spans="1:21" ht="27" hidden="1" customHeight="1">
       <c r="A9" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B9" s="87" t="s">
+      <c r="B9" s="85" t="s">
         <v>1417</v>
       </c>
       <c r="C9" s="3" t="s">
@@ -6863,11 +6869,11 @@
       </c>
       <c r="R9" s="53"/>
     </row>
-    <row r="10" spans="1:21" ht="40.5">
+    <row r="10" spans="1:21" ht="40.5" hidden="1">
       <c r="A10" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B10" s="87" t="s">
+      <c r="B10" s="85" t="s">
         <v>1418</v>
       </c>
       <c r="C10" s="3" t="s">
@@ -6913,11 +6919,11 @@
       </c>
       <c r="R10" s="53"/>
     </row>
-    <row r="11" spans="1:21" ht="43.5">
+    <row r="11" spans="1:21" ht="43.5" hidden="1">
       <c r="A11" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B11" s="87" t="s">
+      <c r="B11" s="85" t="s">
         <v>1419</v>
       </c>
       <c r="C11" s="3" t="s">
@@ -6961,11 +6967,11 @@
       <c r="Q11" s="71"/>
       <c r="R11" s="53"/>
     </row>
-    <row r="12" spans="1:21" ht="67.5" customHeight="1">
+    <row r="12" spans="1:21" ht="67.5" hidden="1" customHeight="1">
       <c r="A12" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B12" s="87" t="s">
+      <c r="B12" s="85" t="s">
         <v>1420</v>
       </c>
       <c r="C12" s="3" t="s">
@@ -7014,7 +7020,7 @@
       <c r="A13" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B13" s="87" t="s">
+      <c r="B13" s="85" t="s">
         <v>1421</v>
       </c>
       <c r="C13" s="3" t="s">
@@ -7062,11 +7068,11 @@
       </c>
       <c r="R13" s="53"/>
     </row>
-    <row r="14" spans="1:21" ht="36.5" customHeight="1">
+    <row r="14" spans="1:21" ht="36.5" hidden="1" customHeight="1">
       <c r="A14" s="51" t="s">
         <v>48</v>
       </c>
-      <c r="B14" s="87" t="s">
+      <c r="B14" s="85" t="s">
         <v>1422</v>
       </c>
       <c r="C14" s="38" t="s">
@@ -7118,11 +7124,11 @@
         <v>1222</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="54">
+    <row r="15" spans="1:21" ht="54" hidden="1">
       <c r="A15" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B15" s="87" t="s">
+      <c r="B15" s="85" t="s">
         <v>1423</v>
       </c>
       <c r="C15" s="38" t="s">
@@ -7169,11 +7175,11 @@
       </c>
       <c r="Q15" s="7"/>
     </row>
-    <row r="16" spans="1:21" ht="27">
+    <row r="16" spans="1:21" ht="27" hidden="1">
       <c r="A16" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B16" s="87" t="s">
+      <c r="B16" s="85" t="s">
         <v>1424</v>
       </c>
       <c r="C16" s="3" t="s">
@@ -7216,11 +7222,11 @@
       </c>
       <c r="Q16" s="7"/>
     </row>
-    <row r="17" spans="1:18">
+    <row r="17" spans="1:18" hidden="1">
       <c r="A17" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B17" s="87" t="s">
+      <c r="B17" s="85" t="s">
         <v>1425</v>
       </c>
       <c r="C17" s="3" t="s">
@@ -7266,11 +7272,11 @@
         <v>47</v>
       </c>
     </row>
-    <row r="18" spans="1:18" ht="40.5">
+    <row r="18" spans="1:18" ht="40.5" hidden="1">
       <c r="A18" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B18" s="87" t="s">
+      <c r="B18" s="85" t="s">
         <v>1426</v>
       </c>
       <c r="C18" s="3" t="s">
@@ -7320,7 +7326,7 @@
       <c r="A19" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B19" s="87" t="s">
+      <c r="B19" s="85" t="s">
         <v>1427</v>
       </c>
       <c r="C19" s="3" t="s">
@@ -7368,11 +7374,11 @@
         <v>1364</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="40.5">
+    <row r="20" spans="1:18" ht="40.5" hidden="1">
       <c r="A20" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B20" s="87" t="s">
+      <c r="B20" s="85" t="s">
         <v>1428</v>
       </c>
       <c r="C20" s="3" t="s">
@@ -7415,11 +7421,11 @@
       </c>
       <c r="R20" s="53"/>
     </row>
-    <row r="21" spans="1:18" ht="40.5">
+    <row r="21" spans="1:18" ht="40.5" hidden="1">
       <c r="A21" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B21" s="87" t="s">
+      <c r="B21" s="85" t="s">
         <v>1429</v>
       </c>
       <c r="C21" s="3" t="s">
@@ -7462,11 +7468,11 @@
       </c>
       <c r="Q21" s="7"/>
     </row>
-    <row r="22" spans="1:18" ht="72.5">
+    <row r="22" spans="1:18" ht="72.5" hidden="1">
       <c r="A22" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B22" s="87" t="s">
+      <c r="B22" s="85" t="s">
         <v>1430</v>
       </c>
       <c r="C22" s="3" t="s">
@@ -7518,11 +7524,11 @@
         <v>1253</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="43.5">
+    <row r="23" spans="1:18" ht="43.5" hidden="1">
       <c r="A23" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="B23" s="87" t="s">
+      <c r="B23" s="85" t="s">
         <v>1431</v>
       </c>
       <c r="C23" s="3" t="s">
@@ -7569,7 +7575,7 @@
       <c r="A24" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="B24" s="87" t="s">
+      <c r="B24" s="85" t="s">
         <v>1432</v>
       </c>
       <c r="C24" s="3" t="s">
@@ -7611,11 +7617,11 @@
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:18">
+    <row r="25" spans="1:18" hidden="1">
       <c r="A25" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B25" s="87" t="s">
+      <c r="B25" s="85" t="s">
         <v>1433</v>
       </c>
       <c r="C25" s="3" t="s">
@@ -7661,11 +7667,11 @@
         <v>47</v>
       </c>
     </row>
-    <row r="26" spans="1:18" ht="27">
+    <row r="26" spans="1:18" ht="27" hidden="1">
       <c r="A26" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B26" s="87" t="s">
+      <c r="B26" s="85" t="s">
         <v>1434</v>
       </c>
       <c r="C26" s="3" t="s">
@@ -7710,11 +7716,11 @@
         <v>1241</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="27">
+    <row r="27" spans="1:18" ht="27" hidden="1">
       <c r="A27" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B27" s="87" t="s">
+      <c r="B27" s="85" t="s">
         <v>1435</v>
       </c>
       <c r="C27" s="3" t="s">
@@ -7757,11 +7763,11 @@
       </c>
       <c r="R27" s="8"/>
     </row>
-    <row r="28" spans="1:18" ht="27">
+    <row r="28" spans="1:18" ht="27" hidden="1">
       <c r="A28" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B28" s="87" t="s">
+      <c r="B28" s="85" t="s">
         <v>1436</v>
       </c>
       <c r="C28" s="3" t="s">
@@ -7813,11 +7819,11 @@
         <v>1231</v>
       </c>
     </row>
-    <row r="29" spans="1:18" ht="40.5">
+    <row r="29" spans="1:18" ht="40.5" hidden="1">
       <c r="A29" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B29" s="87" t="s">
+      <c r="B29" s="85" t="s">
         <v>1437</v>
       </c>
       <c r="C29" s="3" t="s">
@@ -7867,7 +7873,7 @@
       <c r="A30" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B30" s="87" t="s">
+      <c r="B30" s="85" t="s">
         <v>1438</v>
       </c>
       <c r="C30" s="3" t="s">
@@ -7923,7 +7929,7 @@
       <c r="A31" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B31" s="87" t="s">
+      <c r="B31" s="85" t="s">
         <v>1439</v>
       </c>
       <c r="C31" s="3" t="s">
@@ -7975,11 +7981,11 @@
         <v>1334</v>
       </c>
     </row>
-    <row r="32" spans="1:18" ht="58">
+    <row r="32" spans="1:18" ht="58" hidden="1">
       <c r="A32" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B32" s="87" t="s">
+      <c r="B32" s="85" t="s">
         <v>1440</v>
       </c>
       <c r="C32" s="3" t="s">
@@ -8026,7 +8032,7 @@
       <c r="A33" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B33" s="87" t="s">
+      <c r="B33" s="85" t="s">
         <v>1441</v>
       </c>
       <c r="C33" s="3" t="s">
@@ -8078,11 +8084,11 @@
         <v>1236</v>
       </c>
     </row>
-    <row r="34" spans="1:18" ht="27">
+    <row r="34" spans="1:18" ht="27" hidden="1">
       <c r="A34" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B34" s="87" t="s">
+      <c r="B34" s="85" t="s">
         <v>1442</v>
       </c>
       <c r="C34" s="3" t="s">
@@ -8125,11 +8131,11 @@
       </c>
       <c r="Q34" s="7"/>
     </row>
-    <row r="35" spans="1:18" ht="27">
+    <row r="35" spans="1:18" ht="27" hidden="1">
       <c r="A35" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B35" s="87" t="s">
+      <c r="B35" s="85" t="s">
         <v>1443</v>
       </c>
       <c r="C35" s="3" t="s">
@@ -8176,11 +8182,11 @@
       </c>
       <c r="Q35" s="7"/>
     </row>
-    <row r="36" spans="1:18" ht="43.5">
+    <row r="36" spans="1:18" ht="43.5" hidden="1">
       <c r="A36" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B36" s="87" t="s">
+      <c r="B36" s="85" t="s">
         <v>1444</v>
       </c>
       <c r="C36" s="3" t="s">
@@ -8227,11 +8233,11 @@
       </c>
       <c r="Q36" s="7"/>
     </row>
-    <row r="37" spans="1:18">
+    <row r="37" spans="1:18" hidden="1">
       <c r="A37" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B37" s="87" t="s">
+      <c r="B37" s="85" t="s">
         <v>1445</v>
       </c>
       <c r="C37" s="3" t="s">
@@ -8266,11 +8272,11 @@
       </c>
       <c r="O37" s="2"/>
     </row>
-    <row r="38" spans="1:18" s="7" customFormat="1" ht="40.5">
+    <row r="38" spans="1:18" s="7" customFormat="1" ht="40.5" hidden="1">
       <c r="A38" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B38" s="87" t="s">
+      <c r="B38" s="85" t="s">
         <v>1446</v>
       </c>
       <c r="C38" s="3" t="s">
@@ -8312,11 +8318,11 @@
         <v>1212</v>
       </c>
     </row>
-    <row r="39" spans="1:18" ht="29">
+    <row r="39" spans="1:18" ht="29" hidden="1">
       <c r="A39" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B39" s="87" t="s">
+      <c r="B39" s="85" t="s">
         <v>1447</v>
       </c>
       <c r="C39" s="3" t="s">
@@ -8358,11 +8364,11 @@
         <v>1212</v>
       </c>
     </row>
-    <row r="40" spans="1:18" ht="27">
+    <row r="40" spans="1:18" ht="27" hidden="1">
       <c r="A40" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B40" s="87" t="s">
+      <c r="B40" s="85" t="s">
         <v>1448</v>
       </c>
       <c r="C40" s="3" t="s">
@@ -8407,11 +8413,11 @@
         <v>1365</v>
       </c>
     </row>
-    <row r="41" spans="1:18" ht="27">
+    <row r="41" spans="1:18" ht="27" hidden="1">
       <c r="A41" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B41" s="87" t="s">
+      <c r="B41" s="85" t="s">
         <v>1449</v>
       </c>
       <c r="C41" s="3" t="s">
@@ -8456,11 +8462,11 @@
         <v>1367</v>
       </c>
     </row>
-    <row r="42" spans="1:18" ht="43.5">
+    <row r="42" spans="1:18" ht="43.5" hidden="1">
       <c r="A42" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B42" s="87" t="s">
+      <c r="B42" s="85" t="s">
         <v>1450</v>
       </c>
       <c r="C42" s="3" t="s">
@@ -8506,7 +8512,7 @@
       <c r="A43" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B43" s="87" t="s">
+      <c r="B43" s="85" t="s">
         <v>1451</v>
       </c>
       <c r="C43" s="8" t="s">
@@ -8548,11 +8554,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="44" spans="1:18" ht="101.5">
+    <row r="44" spans="1:18" ht="101.5" hidden="1">
       <c r="A44" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B44" s="87" t="s">
+      <c r="B44" s="85" t="s">
         <v>1452</v>
       </c>
       <c r="C44" s="3" t="s">
@@ -8604,11 +8610,11 @@
         <v>1368</v>
       </c>
     </row>
-    <row r="45" spans="1:18" ht="27">
+    <row r="45" spans="1:18" ht="27" hidden="1">
       <c r="A45" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B45" s="87" t="s">
+      <c r="B45" s="85" t="s">
         <v>1453</v>
       </c>
       <c r="C45" s="3" t="s">
@@ -8653,11 +8659,11 @@
         <v>1241</v>
       </c>
     </row>
-    <row r="46" spans="1:18" ht="40.5">
+    <row r="46" spans="1:18" ht="40.5" hidden="1">
       <c r="A46" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B46" s="87" t="s">
+      <c r="B46" s="85" t="s">
         <v>1454</v>
       </c>
       <c r="C46" s="3" t="s">
@@ -8706,11 +8712,11 @@
         <v>1241</v>
       </c>
     </row>
-    <row r="47" spans="1:18" ht="40.5">
+    <row r="47" spans="1:18" ht="40.5" hidden="1">
       <c r="A47" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B47" s="87" t="s">
+      <c r="B47" s="85" t="s">
         <v>1455</v>
       </c>
       <c r="C47" s="3" t="s">
@@ -8745,7 +8751,7 @@
       <c r="A48" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="B48" s="87" t="s">
+      <c r="B48" s="85" t="s">
         <v>1456</v>
       </c>
       <c r="C48" s="3" t="s">
@@ -8791,7 +8797,7 @@
       <c r="A49" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B49" s="87" t="s">
+      <c r="B49" s="85" t="s">
         <v>1457</v>
       </c>
       <c r="C49" s="3" t="s">
@@ -8841,7 +8847,7 @@
       <c r="A50" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B50" s="87" t="s">
+      <c r="B50" s="85" t="s">
         <v>1458</v>
       </c>
       <c r="C50" s="3" t="s">
@@ -8897,7 +8903,7 @@
       <c r="A51" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B51" s="87" t="s">
+      <c r="B51" s="85" t="s">
         <v>1459</v>
       </c>
       <c r="C51" s="3" t="s">
@@ -8943,11 +8949,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="52" spans="1:18" ht="29">
+    <row r="52" spans="1:18" ht="29" hidden="1">
       <c r="A52" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B52" s="87" t="s">
+      <c r="B52" s="85" t="s">
         <v>1460</v>
       </c>
       <c r="C52" s="3" t="s">
@@ -8999,11 +9005,11 @@
         <v>1239</v>
       </c>
     </row>
-    <row r="53" spans="1:18" ht="27">
+    <row r="53" spans="1:18" ht="27" hidden="1">
       <c r="A53" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B53" s="87" t="s">
+      <c r="B53" s="85" t="s">
         <v>1461</v>
       </c>
       <c r="C53" s="3" t="s">
@@ -9043,11 +9049,11 @@
         <v>1400</v>
       </c>
     </row>
-    <row r="54" spans="1:18" ht="49.5">
+    <row r="54" spans="1:18" ht="49.5" hidden="1">
       <c r="A54" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B54" s="87" t="s">
+      <c r="B54" s="85" t="s">
         <v>1462</v>
       </c>
       <c r="C54" s="37" t="s">
@@ -9096,11 +9102,11 @@
         <v>1363</v>
       </c>
     </row>
-    <row r="55" spans="1:18" ht="29">
+    <row r="55" spans="1:18" ht="29" hidden="1">
       <c r="A55" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B55" s="87" t="s">
+      <c r="B55" s="85" t="s">
         <v>1463</v>
       </c>
       <c r="C55" s="3" t="s">
@@ -9146,11 +9152,11 @@
         <v>1241</v>
       </c>
     </row>
-    <row r="56" spans="1:18" ht="29">
+    <row r="56" spans="1:18" ht="29" hidden="1">
       <c r="A56" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B56" s="87" t="s">
+      <c r="B56" s="85" t="s">
         <v>1464</v>
       </c>
       <c r="C56" s="3" t="s">
@@ -9200,11 +9206,11 @@
         <v>1371</v>
       </c>
     </row>
-    <row r="57" spans="1:18" ht="40.5">
+    <row r="57" spans="1:18" ht="40.5" hidden="1">
       <c r="A57" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B57" s="87" t="s">
+      <c r="B57" s="85" t="s">
         <v>1465</v>
       </c>
       <c r="C57" s="3" t="s">
@@ -9257,7 +9263,7 @@
       <c r="A58" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="B58" s="87" t="s">
+      <c r="B58" s="85" t="s">
         <v>1466</v>
       </c>
       <c r="C58" s="3" t="s">
@@ -9299,11 +9305,11 @@
         <v>47</v>
       </c>
     </row>
-    <row r="59" spans="1:18" ht="43.5">
+    <row r="59" spans="1:18" ht="43.5" hidden="1">
       <c r="A59" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B59" s="87" t="s">
+      <c r="B59" s="85" t="s">
         <v>1467</v>
       </c>
       <c r="C59" s="3" t="s">
@@ -9349,11 +9355,11 @@
         <v>1241</v>
       </c>
     </row>
-    <row r="60" spans="1:18" s="7" customFormat="1" ht="27">
+    <row r="60" spans="1:18" s="7" customFormat="1" ht="27" hidden="1">
       <c r="A60" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B60" s="87" t="s">
+      <c r="B60" s="85" t="s">
         <v>1468</v>
       </c>
       <c r="C60" s="3" t="s">
@@ -9392,11 +9398,11 @@
         <v>322</v>
       </c>
     </row>
-    <row r="61" spans="1:18" s="7" customFormat="1" ht="29">
+    <row r="61" spans="1:18" s="7" customFormat="1" ht="29" hidden="1">
       <c r="A61" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B61" s="87" t="s">
+      <c r="B61" s="85" t="s">
         <v>1469</v>
       </c>
       <c r="C61" s="3" t="s">
@@ -9440,11 +9446,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="62" spans="1:18" s="7" customFormat="1" ht="27">
+    <row r="62" spans="1:18" s="7" customFormat="1" ht="27" hidden="1">
       <c r="A62" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B62" s="87" t="s">
+      <c r="B62" s="85" t="s">
         <v>1470</v>
       </c>
       <c r="C62" s="3" t="s">
@@ -9494,7 +9500,7 @@
       <c r="A63" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B63" s="87" t="s">
+      <c r="B63" s="85" t="s">
         <v>1471</v>
       </c>
       <c r="C63" s="3" t="s">
@@ -9544,7 +9550,7 @@
       <c r="A64" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B64" s="87" t="s">
+      <c r="B64" s="85" t="s">
         <v>1472</v>
       </c>
       <c r="C64" s="75" t="s">
@@ -9592,7 +9598,7 @@
       <c r="A65" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B65" s="87" t="s">
+      <c r="B65" s="85" t="s">
         <v>1473</v>
       </c>
       <c r="C65" s="3" t="s">
@@ -9640,11 +9646,11 @@
         <v>1261</v>
       </c>
     </row>
-    <row r="66" spans="1:22" ht="72.5">
+    <row r="66" spans="1:22" ht="72.5" hidden="1">
       <c r="A66" s="9" t="s">
         <v>347</v>
       </c>
-      <c r="B66" s="87" t="s">
+      <c r="B66" s="85" t="s">
         <v>1474</v>
       </c>
       <c r="C66" s="3" t="s">
@@ -9696,11 +9702,11 @@
         <v>1248</v>
       </c>
     </row>
-    <row r="67" spans="1:22" ht="27" customHeight="1">
+    <row r="67" spans="1:22" ht="27" hidden="1" customHeight="1">
       <c r="A67" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B67" s="87" t="s">
+      <c r="B67" s="85" t="s">
         <v>1475</v>
       </c>
       <c r="C67" s="3" t="s">
@@ -9746,11 +9752,11 @@
       <c r="T67" s="4"/>
       <c r="U67" s="5"/>
     </row>
-    <row r="68" spans="1:22" ht="27">
+    <row r="68" spans="1:22" ht="27" hidden="1">
       <c r="A68" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B68" s="87" t="s">
+      <c r="B68" s="85" t="s">
         <v>1476</v>
       </c>
       <c r="C68" s="3" t="s">
@@ -9793,11 +9799,11 @@
       </c>
       <c r="R68" s="8"/>
     </row>
-    <row r="69" spans="1:22" ht="27">
+    <row r="69" spans="1:22" ht="27" hidden="1">
       <c r="A69" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B69" s="87" t="s">
+      <c r="B69" s="85" t="s">
         <v>1477</v>
       </c>
       <c r="C69" s="3" t="s">
@@ -9844,11 +9850,11 @@
       </c>
       <c r="R69" s="8"/>
     </row>
-    <row r="70" spans="1:22">
+    <row r="70" spans="1:22" hidden="1">
       <c r="A70" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B70" s="87" t="s">
+      <c r="B70" s="85" t="s">
         <v>1478</v>
       </c>
       <c r="C70" s="3" t="s">
@@ -9893,11 +9899,11 @@
       <c r="U70" s="4"/>
       <c r="V70" s="3"/>
     </row>
-    <row r="71" spans="1:22" ht="27">
+    <row r="71" spans="1:22" ht="27" hidden="1">
       <c r="A71" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B71" s="87" t="s">
+      <c r="B71" s="85" t="s">
         <v>1479</v>
       </c>
       <c r="C71" s="3" t="s">
@@ -9945,11 +9951,11 @@
       <c r="R71" s="8"/>
       <c r="U71" s="4"/>
     </row>
-    <row r="72" spans="1:22" ht="27">
+    <row r="72" spans="1:22" ht="27" hidden="1">
       <c r="A72" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B72" s="87" t="s">
+      <c r="B72" s="85" t="s">
         <v>1480</v>
       </c>
       <c r="C72" s="3" t="s">
@@ -9994,11 +10000,11 @@
       <c r="R72" s="8"/>
       <c r="U72" s="4"/>
     </row>
-    <row r="73" spans="1:22">
+    <row r="73" spans="1:22" hidden="1">
       <c r="A73" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B73" s="87" t="s">
+      <c r="B73" s="85" t="s">
         <v>1481</v>
       </c>
       <c r="C73" s="3" t="s">
@@ -10046,11 +10052,11 @@
       <c r="R73" s="8"/>
       <c r="U73" s="4"/>
     </row>
-    <row r="74" spans="1:22" ht="27">
+    <row r="74" spans="1:22" ht="27" hidden="1">
       <c r="A74" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B74" s="87" t="s">
+      <c r="B74" s="85" t="s">
         <v>1482</v>
       </c>
       <c r="C74" s="3" t="s">
@@ -10094,11 +10100,11 @@
       <c r="R74" s="8"/>
       <c r="U74" s="4"/>
     </row>
-    <row r="75" spans="1:22" ht="29">
+    <row r="75" spans="1:22" ht="29" hidden="1">
       <c r="A75" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B75" s="87" t="s">
+      <c r="B75" s="85" t="s">
         <v>1483</v>
       </c>
       <c r="C75" s="3" t="s">
@@ -10140,11 +10146,11 @@
       <c r="R75" s="8"/>
       <c r="U75" s="4"/>
     </row>
-    <row r="76" spans="1:22" ht="27">
+    <row r="76" spans="1:22" ht="27" hidden="1">
       <c r="A76" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B76" s="87" t="s">
+      <c r="B76" s="85" t="s">
         <v>1484</v>
       </c>
       <c r="C76" s="3" t="s">
@@ -10185,11 +10191,11 @@
       </c>
       <c r="R76" s="8"/>
     </row>
-    <row r="77" spans="1:22" ht="348">
+    <row r="77" spans="1:22" ht="348" hidden="1">
       <c r="A77" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B77" s="87" t="s">
+      <c r="B77" s="85" t="s">
         <v>1485</v>
       </c>
       <c r="C77" s="3" t="s">
@@ -10238,11 +10244,11 @@
         <v>1250</v>
       </c>
     </row>
-    <row r="78" spans="1:22" ht="27">
+    <row r="78" spans="1:22" ht="27" hidden="1">
       <c r="A78" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B78" s="87" t="s">
+      <c r="B78" s="85" t="s">
         <v>1486</v>
       </c>
       <c r="C78" s="3" t="s">
@@ -10289,11 +10295,11 @@
       </c>
       <c r="R78" s="8"/>
     </row>
-    <row r="79" spans="1:22" ht="27">
+    <row r="79" spans="1:22" ht="27" hidden="1">
       <c r="A79" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B79" s="87" t="s">
+      <c r="B79" s="85" t="s">
         <v>1487</v>
       </c>
       <c r="C79" s="3" t="s">
@@ -10334,11 +10340,11 @@
       </c>
       <c r="R79" s="8"/>
     </row>
-    <row r="80" spans="1:22" ht="27">
+    <row r="80" spans="1:22" ht="40.5" hidden="1">
       <c r="A80" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B80" s="87" t="s">
+      <c r="B80" s="85" t="s">
         <v>1488</v>
       </c>
       <c r="C80" s="3" t="s">
@@ -10381,11 +10387,11 @@
       </c>
       <c r="R80" s="8"/>
     </row>
-    <row r="81" spans="1:18" ht="40.5">
+    <row r="81" spans="1:18" ht="40.5" hidden="1">
       <c r="A81" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B81" s="87" t="s">
+      <c r="B81" s="85" t="s">
         <v>1489</v>
       </c>
       <c r="C81" s="3" t="s">
@@ -10422,11 +10428,11 @@
       </c>
       <c r="R81" s="8"/>
     </row>
-    <row r="82" spans="1:18" ht="40.5">
+    <row r="82" spans="1:18" ht="40.5" hidden="1">
       <c r="A82" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B82" s="87" t="s">
+      <c r="B82" s="85" t="s">
         <v>1490</v>
       </c>
       <c r="C82" s="3" t="s">
@@ -10467,11 +10473,11 @@
       </c>
       <c r="R82" s="8"/>
     </row>
-    <row r="83" spans="1:18" ht="40.5">
+    <row r="83" spans="1:18" ht="40.5" hidden="1">
       <c r="A83" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B83" s="87" t="s">
+      <c r="B83" s="85" t="s">
         <v>1491</v>
       </c>
       <c r="C83" s="3" t="s">
@@ -10518,11 +10524,11 @@
       </c>
       <c r="R83" s="8"/>
     </row>
-    <row r="84" spans="1:18" ht="27">
+    <row r="84" spans="1:18" ht="27" hidden="1">
       <c r="A84" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B84" s="87" t="s">
+      <c r="B84" s="85" t="s">
         <v>1492</v>
       </c>
       <c r="C84" s="3" t="s">
@@ -10569,11 +10575,11 @@
       </c>
       <c r="R84" s="8"/>
     </row>
-    <row r="85" spans="1:18" ht="27">
+    <row r="85" spans="1:18" ht="27" hidden="1">
       <c r="A85" s="9" t="s">
         <v>434</v>
       </c>
-      <c r="B85" s="87" t="s">
+      <c r="B85" s="85" t="s">
         <v>1493</v>
       </c>
       <c r="C85" s="3" t="s">
@@ -10620,11 +10626,11 @@
       </c>
       <c r="R85" s="8"/>
     </row>
-    <row r="86" spans="1:18">
+    <row r="86" spans="1:18" hidden="1">
       <c r="A86" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B86" s="87" t="s">
+      <c r="B86" s="85" t="s">
         <v>1494</v>
       </c>
       <c r="C86" s="3" t="s">
@@ -10667,11 +10673,11 @@
       </c>
       <c r="R86" s="8"/>
     </row>
-    <row r="87" spans="1:18" ht="27">
+    <row r="87" spans="1:18" ht="27" hidden="1">
       <c r="A87" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B87" s="87" t="s">
+      <c r="B87" s="85" t="s">
         <v>1495</v>
       </c>
       <c r="C87" s="3" t="s">
@@ -10715,11 +10721,11 @@
       </c>
       <c r="R87" s="8"/>
     </row>
-    <row r="88" spans="1:18" ht="43.5">
+    <row r="88" spans="1:18" ht="43.5" hidden="1">
       <c r="A88" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B88" s="87" t="s">
+      <c r="B88" s="85" t="s">
         <v>1496</v>
       </c>
       <c r="C88" s="3" t="s">
@@ -10766,7 +10772,7 @@
       <c r="A89" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B89" s="87" t="s">
+      <c r="B89" s="85" t="s">
         <v>1497</v>
       </c>
       <c r="C89" s="3" t="s">
@@ -10803,11 +10809,11 @@
       </c>
       <c r="R89" s="8"/>
     </row>
-    <row r="90" spans="1:18" ht="29">
+    <row r="90" spans="1:18" ht="29" hidden="1">
       <c r="A90" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="B90" s="87" t="s">
+      <c r="B90" s="85" t="s">
         <v>1498</v>
       </c>
       <c r="C90" s="3" t="s">
@@ -10850,11 +10856,11 @@
       </c>
       <c r="R90" s="8"/>
     </row>
-    <row r="91" spans="1:18" ht="27">
+    <row r="91" spans="1:18" ht="27" hidden="1">
       <c r="A91" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B91" s="87" t="s">
+      <c r="B91" s="85" t="s">
         <v>1499</v>
       </c>
       <c r="C91" s="3" t="s">
@@ -10896,11 +10902,11 @@
         <v>47</v>
       </c>
     </row>
-    <row r="92" spans="1:18" ht="27">
+    <row r="92" spans="1:18" ht="27" hidden="1">
       <c r="A92" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B92" s="87" t="s">
+      <c r="B92" s="85" t="s">
         <v>1500</v>
       </c>
       <c r="C92" s="3" t="s">
@@ -10938,7 +10944,7 @@
       <c r="A93" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B93" s="87" t="s">
+      <c r="B93" s="85" t="s">
         <v>1501</v>
       </c>
       <c r="C93" s="3" t="s">
@@ -10975,11 +10981,11 @@
         <v>475</v>
       </c>
     </row>
-    <row r="94" spans="1:18" ht="29">
+    <row r="94" spans="1:18" ht="29" hidden="1">
       <c r="A94" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B94" s="87" t="s">
+      <c r="B94" s="85" t="s">
         <v>1502</v>
       </c>
       <c r="C94" s="3" t="s">
@@ -11019,11 +11025,11 @@
         <v>94</v>
       </c>
     </row>
-    <row r="95" spans="1:18" ht="40.5">
+    <row r="95" spans="1:18" ht="40.5" hidden="1">
       <c r="A95" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B95" s="87" t="s">
+      <c r="B95" s="85" t="s">
         <v>1503</v>
       </c>
       <c r="C95" s="3" t="s">
@@ -11063,11 +11069,11 @@
         <v>480</v>
       </c>
     </row>
-    <row r="96" spans="1:18" ht="29">
+    <row r="96" spans="1:18" ht="29" hidden="1">
       <c r="A96" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B96" s="87" t="s">
+      <c r="B96" s="85" t="s">
         <v>1504</v>
       </c>
       <c r="C96" s="3" t="s">
@@ -11109,11 +11115,11 @@
         <v>47</v>
       </c>
     </row>
-    <row r="97" spans="1:21" ht="27">
+    <row r="97" spans="1:21" ht="27" hidden="1">
       <c r="A97" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B97" s="87" t="s">
+      <c r="B97" s="85" t="s">
         <v>1505</v>
       </c>
       <c r="C97" s="3" t="s">
@@ -11162,11 +11168,11 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="98" spans="1:21" ht="27">
+    <row r="98" spans="1:21" ht="27" hidden="1">
       <c r="A98" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B98" s="87" t="s">
+      <c r="B98" s="85" t="s">
         <v>1506</v>
       </c>
       <c r="C98" s="3" t="s">
@@ -11203,11 +11209,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="99" spans="1:21" ht="27">
+    <row r="99" spans="1:21" ht="27" hidden="1">
       <c r="A99" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B99" s="87" t="s">
+      <c r="B99" s="85" t="s">
         <v>1507</v>
       </c>
       <c r="C99" s="3" t="s">
@@ -11253,11 +11259,11 @@
         <v>47</v>
       </c>
     </row>
-    <row r="100" spans="1:21" ht="40.5">
+    <row r="100" spans="1:21" ht="40.5" hidden="1">
       <c r="A100" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B100" s="87" t="s">
+      <c r="B100" s="85" t="s">
         <v>1508</v>
       </c>
       <c r="C100" s="3" t="s">
@@ -11297,11 +11303,11 @@
         <v>504</v>
       </c>
     </row>
-    <row r="101" spans="1:21" ht="29">
+    <row r="101" spans="1:21" ht="29" hidden="1">
       <c r="A101" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B101" s="87" t="s">
+      <c r="B101" s="85" t="s">
         <v>1509</v>
       </c>
       <c r="C101" s="3" t="s">
@@ -11343,11 +11349,11 @@
         <v>47</v>
       </c>
     </row>
-    <row r="102" spans="1:21" ht="40.5">
+    <row r="102" spans="1:21" ht="40.5" hidden="1">
       <c r="A102" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B102" s="87" t="s">
+      <c r="B102" s="85" t="s">
         <v>1510</v>
       </c>
       <c r="C102" s="3" t="s">
@@ -11389,11 +11395,11 @@
         <v>47</v>
       </c>
     </row>
-    <row r="103" spans="1:21" ht="27">
+    <row r="103" spans="1:21" ht="27" hidden="1">
       <c r="A103" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B103" s="87" t="s">
+      <c r="B103" s="85" t="s">
         <v>1511</v>
       </c>
       <c r="C103" s="3" t="s">
@@ -11445,11 +11451,11 @@
         <v>1344</v>
       </c>
     </row>
-    <row r="104" spans="1:21" ht="29">
+    <row r="104" spans="1:21" ht="29" hidden="1">
       <c r="A104" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="B104" s="87" t="s">
+      <c r="B104" s="85" t="s">
         <v>1512</v>
       </c>
       <c r="C104" s="3" t="s">
@@ -11491,11 +11497,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="105" spans="1:21" ht="27">
+    <row r="105" spans="1:21" ht="27" hidden="1">
       <c r="A105" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B105" s="87" t="s">
+      <c r="B105" s="85" t="s">
         <v>1513</v>
       </c>
       <c r="C105" s="3" t="s">
@@ -11541,11 +11547,11 @@
         <v>47</v>
       </c>
     </row>
-    <row r="106" spans="1:21" ht="54">
+    <row r="106" spans="1:21" ht="54" hidden="1">
       <c r="A106" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B106" s="87" t="s">
+      <c r="B106" s="85" t="s">
         <v>1514</v>
       </c>
       <c r="C106" s="3" t="s">
@@ -11585,11 +11591,11 @@
         <v>532</v>
       </c>
     </row>
-    <row r="107" spans="1:21" ht="29">
+    <row r="107" spans="1:21" ht="29" hidden="1">
       <c r="A107" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="B107" s="87" t="s">
+      <c r="B107" s="85" t="s">
         <v>1515</v>
       </c>
       <c r="C107" s="3" t="s">
@@ -11640,7 +11646,7 @@
       <c r="A108" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B108" s="87" t="s">
+      <c r="B108" s="85" t="s">
         <v>1516</v>
       </c>
       <c r="C108" s="3" t="s">
@@ -11685,11 +11691,11 @@
       <c r="T108" s="4"/>
       <c r="U108" s="6"/>
     </row>
-    <row r="109" spans="1:21" ht="29">
+    <row r="109" spans="1:21" ht="29" hidden="1">
       <c r="A109" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="B109" s="87" t="s">
+      <c r="B109" s="85" t="s">
         <v>1517</v>
       </c>
       <c r="C109" s="3" t="s">
@@ -11737,11 +11743,11 @@
         <v>1263</v>
       </c>
     </row>
-    <row r="110" spans="1:21" ht="40.5">
+    <row r="110" spans="1:21" ht="40.5" hidden="1">
       <c r="A110" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B110" s="87" t="s">
+      <c r="B110" s="85" t="s">
         <v>1518</v>
       </c>
       <c r="C110" s="3" t="s">
@@ -11793,11 +11799,11 @@
         <v>1255</v>
       </c>
     </row>
-    <row r="111" spans="1:21" ht="27">
+    <row r="111" spans="1:21" ht="27" hidden="1">
       <c r="A111" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="B111" s="87" t="s">
+      <c r="B111" s="85" t="s">
         <v>1519</v>
       </c>
       <c r="C111" s="3" t="s">
@@ -11839,11 +11845,11 @@
         <v>47</v>
       </c>
     </row>
-    <row r="112" spans="1:21" ht="27">
+    <row r="112" spans="1:21" ht="27" hidden="1">
       <c r="A112" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B112" s="87" t="s">
+      <c r="B112" s="85" t="s">
         <v>1520</v>
       </c>
       <c r="C112" s="3" t="s">
@@ -11879,11 +11885,11 @@
         <v>559</v>
       </c>
     </row>
-    <row r="113" spans="1:18" ht="40.5">
+    <row r="113" spans="1:18" ht="40.5" hidden="1">
       <c r="A113" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B113" s="87" t="s">
+      <c r="B113" s="85" t="s">
         <v>1521</v>
       </c>
       <c r="C113" s="3" t="s">
@@ -11922,11 +11928,11 @@
         <v>47</v>
       </c>
     </row>
-    <row r="114" spans="1:18">
+    <row r="114" spans="1:18" hidden="1">
       <c r="A114" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="B114" s="87" t="s">
+      <c r="B114" s="85" t="s">
         <v>1522</v>
       </c>
       <c r="C114" s="3" t="s">
@@ -11972,11 +11978,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="115" spans="1:18" ht="40.5">
+    <row r="115" spans="1:18" ht="40.5" hidden="1">
       <c r="A115" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B115" s="87" t="s">
+      <c r="B115" s="85" t="s">
         <v>1523</v>
       </c>
       <c r="C115" s="3" t="s">
@@ -12016,11 +12022,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="116" spans="1:18" ht="27">
+    <row r="116" spans="1:18" ht="27" hidden="1">
       <c r="A116" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B116" s="87" t="s">
+      <c r="B116" s="85" t="s">
         <v>1524</v>
       </c>
       <c r="C116" s="3" t="s">
@@ -12066,11 +12072,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="117" spans="1:18">
+    <row r="117" spans="1:18" hidden="1">
       <c r="A117" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B117" s="87" t="s">
+      <c r="B117" s="85" t="s">
         <v>1525</v>
       </c>
       <c r="C117" s="3" t="s">
@@ -12112,11 +12118,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="118" spans="1:18" ht="29">
+    <row r="118" spans="1:18" ht="29" hidden="1">
       <c r="A118" s="51" t="s">
         <v>48</v>
       </c>
-      <c r="B118" s="87" t="s">
+      <c r="B118" s="85" t="s">
         <v>1526</v>
       </c>
       <c r="C118" s="38" t="s">
@@ -12164,11 +12170,11 @@
         <v>1259</v>
       </c>
     </row>
-    <row r="119" spans="1:18">
+    <row r="119" spans="1:18" hidden="1">
       <c r="A119" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B119" s="87" t="s">
+      <c r="B119" s="85" t="s">
         <v>1527</v>
       </c>
       <c r="C119" s="3" t="s">
@@ -12210,11 +12216,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="120" spans="1:18" ht="27">
+    <row r="120" spans="1:18" ht="27" hidden="1">
       <c r="A120" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B120" s="87" t="s">
+      <c r="B120" s="85" t="s">
         <v>1528</v>
       </c>
       <c r="C120" s="3" t="s">
@@ -12260,11 +12266,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="121" spans="1:18" ht="27">
+    <row r="121" spans="1:18" ht="27" hidden="1">
       <c r="A121" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B121" s="87" t="s">
+      <c r="B121" s="85" t="s">
         <v>1529</v>
       </c>
       <c r="C121" s="3" t="s">
@@ -12300,11 +12306,11 @@
         <v>604</v>
       </c>
     </row>
-    <row r="122" spans="1:18" ht="27">
+    <row r="122" spans="1:18" ht="27" hidden="1">
       <c r="A122" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B122" s="87" t="s">
+      <c r="B122" s="85" t="s">
         <v>1530</v>
       </c>
       <c r="C122" s="3" t="s">
@@ -12348,7 +12354,7 @@
       <c r="A123" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B123" s="87" t="s">
+      <c r="B123" s="85" t="s">
         <v>1531</v>
       </c>
       <c r="C123" s="3" t="s">
@@ -12391,11 +12397,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="124" spans="1:18" ht="43.5">
+    <row r="124" spans="1:18" ht="43.5" hidden="1">
       <c r="A124" s="35" t="s">
         <v>263</v>
       </c>
-      <c r="B124" s="87" t="s">
+      <c r="B124" s="85" t="s">
         <v>1532</v>
       </c>
       <c r="C124" s="3" t="s">
@@ -12441,11 +12447,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="125" spans="1:18" ht="27">
+    <row r="125" spans="1:18" ht="27" hidden="1">
       <c r="A125" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B125" s="87" t="s">
+      <c r="B125" s="85" t="s">
         <v>1533</v>
       </c>
       <c r="C125" s="38" t="s">
@@ -12497,11 +12503,11 @@
         <v>1267</v>
       </c>
     </row>
-    <row r="126" spans="1:18">
+    <row r="126" spans="1:18" hidden="1">
       <c r="A126" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B126" s="87" t="s">
+      <c r="B126" s="85" t="s">
         <v>1534</v>
       </c>
       <c r="C126" s="3" t="s">
@@ -12553,11 +12559,11 @@
         <v>1316</v>
       </c>
     </row>
-    <row r="127" spans="1:18" ht="27">
+    <row r="127" spans="1:18" ht="27" hidden="1">
       <c r="A127" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B127" s="87" t="s">
+      <c r="B127" s="85" t="s">
         <v>1535</v>
       </c>
       <c r="C127" s="3" t="s">
@@ -12603,11 +12609,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="128" spans="1:18" ht="27">
+    <row r="128" spans="1:18" ht="27" hidden="1">
       <c r="A128" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B128" s="87" t="s">
+      <c r="B128" s="85" t="s">
         <v>1536</v>
       </c>
       <c r="C128" s="3" t="s">
@@ -12653,11 +12659,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="129" spans="1:18" ht="27">
+    <row r="129" spans="1:18" ht="27" hidden="1">
       <c r="A129" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B129" s="87" t="s">
+      <c r="B129" s="85" t="s">
         <v>1537</v>
       </c>
       <c r="C129" s="3" t="s">
@@ -12707,7 +12713,7 @@
       <c r="A130" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B130" s="87" t="s">
+      <c r="B130" s="85" t="s">
         <v>1538</v>
       </c>
       <c r="C130" s="3" t="s">
@@ -12753,11 +12759,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="131" spans="1:18" ht="27">
+    <row r="131" spans="1:18" ht="27" hidden="1">
       <c r="A131" s="47" t="s">
         <v>39</v>
       </c>
-      <c r="B131" s="87" t="s">
+      <c r="B131" s="85" t="s">
         <v>1539</v>
       </c>
       <c r="C131" s="38" t="s">
@@ -12803,11 +12809,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="132" spans="1:18" ht="54">
+    <row r="132" spans="1:18" ht="54" hidden="1">
       <c r="A132" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B132" s="87" t="s">
+      <c r="B132" s="85" t="s">
         <v>1540</v>
       </c>
       <c r="C132" s="38" t="s">
@@ -12850,11 +12856,11 @@
         <v>655</v>
       </c>
     </row>
-    <row r="133" spans="1:18" ht="27">
+    <row r="133" spans="1:18" ht="27" hidden="1">
       <c r="A133" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="B133" s="87" t="s">
+      <c r="B133" s="85" t="s">
         <v>1541</v>
       </c>
       <c r="C133" s="38" t="s">
@@ -12902,11 +12908,11 @@
         <v>1318</v>
       </c>
     </row>
-    <row r="134" spans="1:18" ht="29">
+    <row r="134" spans="1:18" ht="29" hidden="1">
       <c r="A134" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B134" s="87" t="s">
+      <c r="B134" s="85" t="s">
         <v>1542</v>
       </c>
       <c r="C134" s="3" t="s">
@@ -12958,11 +12964,11 @@
         <v>1312</v>
       </c>
     </row>
-    <row r="135" spans="1:18" ht="40.5">
+    <row r="135" spans="1:18" ht="40.5" hidden="1">
       <c r="A135" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B135" s="87" t="s">
+      <c r="B135" s="85" t="s">
         <v>1543</v>
       </c>
       <c r="C135" s="3" t="s">
@@ -13008,7 +13014,7 @@
       <c r="A136" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B136" s="87" t="s">
+      <c r="B136" s="85" t="s">
         <v>1544</v>
       </c>
       <c r="C136" s="3" t="s">
@@ -13056,11 +13062,11 @@
         <v>1269</v>
       </c>
     </row>
-    <row r="137" spans="1:18" ht="27">
+    <row r="137" spans="1:18" ht="27" hidden="1">
       <c r="A137" s="14" t="s">
         <v>676</v>
       </c>
-      <c r="B137" s="87" t="s">
+      <c r="B137" s="85" t="s">
         <v>1545</v>
       </c>
       <c r="C137" s="3" t="s">
@@ -13096,11 +13102,11 @@
         <v>680</v>
       </c>
     </row>
-    <row r="138" spans="1:18" ht="43.5">
+    <row r="138" spans="1:18" ht="43.5" hidden="1">
       <c r="A138" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B138" s="87" t="s">
+      <c r="B138" s="85" t="s">
         <v>1546</v>
       </c>
       <c r="C138" s="3" t="s">
@@ -13150,7 +13156,7 @@
       <c r="A139" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B139" s="87" t="s">
+      <c r="B139" s="85" t="s">
         <v>1547</v>
       </c>
       <c r="C139" s="3" t="s">
@@ -13183,11 +13189,11 @@
         <v>689</v>
       </c>
     </row>
-    <row r="140" spans="1:18" ht="43.5">
+    <row r="140" spans="1:18" ht="43.5" hidden="1">
       <c r="A140" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B140" s="87" t="s">
+      <c r="B140" s="85" t="s">
         <v>1548</v>
       </c>
       <c r="C140" s="3" t="s">
@@ -13224,11 +13230,11 @@
         <v>693</v>
       </c>
     </row>
-    <row r="141" spans="1:18" ht="40.5">
+    <row r="141" spans="1:18" ht="40.5" hidden="1">
       <c r="A141" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B141" s="87" t="s">
+      <c r="B141" s="85" t="s">
         <v>1549</v>
       </c>
       <c r="C141" s="3" t="s">
@@ -13270,11 +13276,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="142" spans="1:18" ht="27">
+    <row r="142" spans="1:18" ht="27" hidden="1">
       <c r="A142" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B142" s="87" t="s">
+      <c r="B142" s="85" t="s">
         <v>1550</v>
       </c>
       <c r="C142" s="3" t="s">
@@ -13326,11 +13332,11 @@
         <v>1270</v>
       </c>
     </row>
-    <row r="143" spans="1:18" ht="27">
+    <row r="143" spans="1:18" ht="27" hidden="1">
       <c r="A143" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B143" s="87" t="s">
+      <c r="B143" s="85" t="s">
         <v>1551</v>
       </c>
       <c r="C143" s="3" t="s">
@@ -13367,7 +13373,7 @@
       <c r="A144" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B144" s="87" t="s">
+      <c r="B144" s="85" t="s">
         <v>1552</v>
       </c>
       <c r="C144" s="3" t="s">
@@ -13409,11 +13415,11 @@
         <v>47</v>
       </c>
     </row>
-    <row r="145" spans="1:18" ht="27">
+    <row r="145" spans="1:18" ht="27" hidden="1">
       <c r="A145" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B145" s="87" t="s">
+      <c r="B145" s="85" t="s">
         <v>1553</v>
       </c>
       <c r="C145" s="3" t="s">
@@ -13446,11 +13452,11 @@
         <v>716</v>
       </c>
     </row>
-    <row r="146" spans="1:18">
+    <row r="146" spans="1:18" hidden="1">
       <c r="A146" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B146" s="87" t="s">
+      <c r="B146" s="85" t="s">
         <v>1554</v>
       </c>
       <c r="C146" s="3" t="s">
@@ -13496,11 +13502,11 @@
         <v>47</v>
       </c>
     </row>
-    <row r="147" spans="1:18" ht="40.5">
+    <row r="147" spans="1:18" ht="40.5" hidden="1">
       <c r="A147" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B147" s="87" t="s">
+      <c r="B147" s="85" t="s">
         <v>1555</v>
       </c>
       <c r="C147" s="3" t="s">
@@ -13552,11 +13558,11 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="148" spans="1:18" ht="27">
+    <row r="148" spans="1:18" ht="27" hidden="1">
       <c r="A148" s="48" t="s">
         <v>158</v>
       </c>
-      <c r="B148" s="87" t="s">
+      <c r="B148" s="85" t="s">
         <v>1556</v>
       </c>
       <c r="C148" s="39" t="s">
@@ -13602,7 +13608,7 @@
       <c r="A149" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B149" s="87" t="s">
+      <c r="B149" s="85" t="s">
         <v>1557</v>
       </c>
       <c r="C149" s="41" t="s">
@@ -13635,11 +13641,11 @@
         <v>735</v>
       </c>
     </row>
-    <row r="150" spans="1:18" ht="29">
+    <row r="150" spans="1:18" ht="29" hidden="1">
       <c r="A150" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B150" s="87" t="s">
+      <c r="B150" s="85" t="s">
         <v>1558</v>
       </c>
       <c r="C150" s="3" t="s">
@@ -13685,11 +13691,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="151" spans="1:18" ht="43.5">
+    <row r="151" spans="1:18" ht="43.5" hidden="1">
       <c r="A151" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B151" s="87" t="s">
+      <c r="B151" s="85" t="s">
         <v>1559</v>
       </c>
       <c r="C151" s="3" t="s">
@@ -13735,7 +13741,7 @@
       <c r="A152" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B152" s="87" t="s">
+      <c r="B152" s="85" t="s">
         <v>1560</v>
       </c>
       <c r="C152" s="3" t="s">
@@ -13787,11 +13793,11 @@
         <v>1314</v>
       </c>
     </row>
-    <row r="153" spans="1:18" ht="27">
+    <row r="153" spans="1:18" ht="27" hidden="1">
       <c r="A153" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B153" s="87" t="s">
+      <c r="B153" s="85" t="s">
         <v>1561</v>
       </c>
       <c r="C153" s="3" t="s">
@@ -13837,11 +13843,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="154" spans="1:18">
+    <row r="154" spans="1:18" hidden="1">
       <c r="A154" s="82" t="s">
         <v>48</v>
       </c>
-      <c r="B154" s="87" t="s">
+      <c r="B154" s="85" t="s">
         <v>1562</v>
       </c>
       <c r="C154" s="3" t="s">
@@ -13873,11 +13879,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="155" spans="1:18" ht="43.5">
+    <row r="155" spans="1:18" ht="43.5" hidden="1">
       <c r="A155" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B155" s="87" t="s">
+      <c r="B155" s="85" t="s">
         <v>1563</v>
       </c>
       <c r="C155" s="3" t="s">
@@ -13923,11 +13929,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="156" spans="1:18" ht="29">
+    <row r="156" spans="1:18" ht="29" hidden="1">
       <c r="A156" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B156" s="87" t="s">
+      <c r="B156" s="85" t="s">
         <v>1564</v>
       </c>
       <c r="C156" s="3" t="s">
@@ -13973,7 +13979,7 @@
       <c r="A157" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B157" s="87" t="s">
+      <c r="B157" s="85" t="s">
         <v>1565</v>
       </c>
       <c r="C157" s="3" t="s">
@@ -14016,11 +14022,11 @@
         <v>1212</v>
       </c>
     </row>
-    <row r="158" spans="1:18" ht="29">
+    <row r="158" spans="1:18" ht="29" hidden="1">
       <c r="A158" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B158" s="87" t="s">
+      <c r="B158" s="85" t="s">
         <v>1566</v>
       </c>
       <c r="C158" s="3" t="s">
@@ -14062,11 +14068,11 @@
         <v>47</v>
       </c>
     </row>
-    <row r="159" spans="1:18" ht="27">
+    <row r="159" spans="1:18" ht="27" hidden="1">
       <c r="A159" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B159" s="87" t="s">
+      <c r="B159" s="85" t="s">
         <v>1567</v>
       </c>
       <c r="C159" s="3" t="s">
@@ -14108,11 +14114,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="160" spans="1:18" ht="27">
+    <row r="160" spans="1:18" ht="27" hidden="1">
       <c r="A160" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B160" s="87" t="s">
+      <c r="B160" s="85" t="s">
         <v>1568</v>
       </c>
       <c r="C160" s="3" t="s">
@@ -14151,11 +14157,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="161" spans="1:18" ht="54">
+    <row r="161" spans="1:18" ht="54" hidden="1">
       <c r="A161" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B161" s="87" t="s">
+      <c r="B161" s="85" t="s">
         <v>1569</v>
       </c>
       <c r="C161" s="3" t="s">
@@ -14197,7 +14203,7 @@
       <c r="A162" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B162" s="87" t="s">
+      <c r="B162" s="85" t="s">
         <v>1570</v>
       </c>
       <c r="C162" s="3" t="s">
@@ -14249,11 +14255,11 @@
         <v>1320</v>
       </c>
     </row>
-    <row r="163" spans="1:18" ht="43.5">
+    <row r="163" spans="1:18" ht="43.5" hidden="1">
       <c r="A163" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B163" s="87" t="s">
+      <c r="B163" s="85" t="s">
         <v>1571</v>
       </c>
       <c r="C163" s="3" t="s">
@@ -14302,11 +14308,11 @@
         <v>1241</v>
       </c>
     </row>
-    <row r="164" spans="1:18" ht="29">
+    <row r="164" spans="1:18" ht="29" hidden="1">
       <c r="A164" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B164" s="87" t="s">
+      <c r="B164" s="85" t="s">
         <v>1572</v>
       </c>
       <c r="C164" s="3" t="s">
@@ -14349,11 +14355,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="165" spans="1:18" ht="54">
+    <row r="165" spans="1:18" ht="54" hidden="1">
       <c r="A165" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B165" s="87" t="s">
+      <c r="B165" s="85" t="s">
         <v>1573</v>
       </c>
       <c r="C165" s="3" t="s">
@@ -14397,11 +14403,11 @@
         <v>1322</v>
       </c>
     </row>
-    <row r="166" spans="1:18" ht="43.5">
+    <row r="166" spans="1:18" ht="43.5" hidden="1">
       <c r="A166" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B166" s="87" t="s">
+      <c r="B166" s="85" t="s">
         <v>1574</v>
       </c>
       <c r="C166" s="3" t="s">
@@ -14447,11 +14453,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="167" spans="1:18" ht="27">
+    <row r="167" spans="1:18" ht="27" hidden="1">
       <c r="A167" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B167" s="87" t="s">
+      <c r="B167" s="85" t="s">
         <v>1575</v>
       </c>
       <c r="C167" s="3" t="s">
@@ -14492,7 +14498,7 @@
       <c r="A168" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B168" s="87" t="s">
+      <c r="B168" s="85" t="s">
         <v>1576</v>
       </c>
       <c r="C168" s="75" t="s">
@@ -14530,11 +14536,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="169" spans="1:18" ht="40.5">
+    <row r="169" spans="1:18" ht="40.5" hidden="1">
       <c r="A169" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B169" s="87" t="s">
+      <c r="B169" s="85" t="s">
         <v>1577</v>
       </c>
       <c r="C169" s="3" t="s">
@@ -14577,11 +14583,11 @@
         <v>820</v>
       </c>
     </row>
-    <row r="170" spans="1:18" ht="27">
+    <row r="170" spans="1:18" ht="27" hidden="1">
       <c r="A170" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B170" s="87" t="s">
+      <c r="B170" s="85" t="s">
         <v>1578</v>
       </c>
       <c r="C170" s="3" t="s">
@@ -14620,11 +14626,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="171" spans="1:18" ht="29">
+    <row r="171" spans="1:18" ht="29" hidden="1">
       <c r="A171" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B171" s="87" t="s">
+      <c r="B171" s="85" t="s">
         <v>1579</v>
       </c>
       <c r="C171" s="3" t="s">
@@ -14670,7 +14676,7 @@
       <c r="A172" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B172" s="87" t="s">
+      <c r="B172" s="85" t="s">
         <v>1580</v>
       </c>
       <c r="C172" s="3" t="s">
@@ -14717,7 +14723,7 @@
       <c r="A173" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B173" s="87" t="s">
+      <c r="B173" s="85" t="s">
         <v>1581</v>
       </c>
       <c r="C173" s="3" t="s">
@@ -14763,11 +14769,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="174" spans="1:18" ht="27">
+    <row r="174" spans="1:18" ht="27" hidden="1">
       <c r="A174" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B174" s="87" t="s">
+      <c r="B174" s="85" t="s">
         <v>1582</v>
       </c>
       <c r="C174" s="3" t="s">
@@ -14813,11 +14819,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="175" spans="1:18" ht="27">
+    <row r="175" spans="1:18" ht="27" hidden="1">
       <c r="A175" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B175" s="87" t="s">
+      <c r="B175" s="85" t="s">
         <v>1583</v>
       </c>
       <c r="C175" s="3" t="s">
@@ -14856,11 +14862,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="176" spans="1:18" ht="29">
+    <row r="176" spans="1:18" ht="29" hidden="1">
       <c r="A176" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B176" s="87" t="s">
+      <c r="B176" s="85" t="s">
         <v>1584</v>
       </c>
       <c r="C176" s="3" t="s">
@@ -14903,11 +14909,11 @@
         <v>854</v>
       </c>
     </row>
-    <row r="177" spans="1:18" ht="27">
+    <row r="177" spans="1:18" ht="27" hidden="1">
       <c r="A177" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B177" s="87" t="s">
+      <c r="B177" s="85" t="s">
         <v>1585</v>
       </c>
       <c r="C177" s="3" t="s">
@@ -14953,11 +14959,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="178" spans="1:18">
+    <row r="178" spans="1:18" hidden="1">
       <c r="A178" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B178" s="87" t="s">
+      <c r="B178" s="85" t="s">
         <v>1586</v>
       </c>
       <c r="C178" s="75" t="s">
@@ -14997,11 +15003,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="179" spans="1:18">
+    <row r="179" spans="1:18" hidden="1">
       <c r="A179" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B179" s="87" t="s">
+      <c r="B179" s="85" t="s">
         <v>1587</v>
       </c>
       <c r="C179" s="3" t="s">
@@ -15047,11 +15053,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="180" spans="1:18" ht="29">
+    <row r="180" spans="1:18" ht="29" hidden="1">
       <c r="A180" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B180" s="87" t="s">
+      <c r="B180" s="85" t="s">
         <v>1588</v>
       </c>
       <c r="C180" s="3" t="s">
@@ -15097,11 +15103,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="181" spans="1:18" ht="27">
+    <row r="181" spans="1:18" ht="27" hidden="1">
       <c r="A181" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B181" s="87" t="s">
+      <c r="B181" s="85" t="s">
         <v>1589</v>
       </c>
       <c r="C181" s="3" t="s">
@@ -15144,11 +15150,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="182" spans="1:18" ht="27">
+    <row r="182" spans="1:18" ht="27" hidden="1">
       <c r="A182" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B182" s="87" t="s">
+      <c r="B182" s="85" t="s">
         <v>1590</v>
       </c>
       <c r="C182" s="3" t="s">
@@ -15190,11 +15196,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="183" spans="1:18" ht="29">
+    <row r="183" spans="1:18" ht="29" hidden="1">
       <c r="A183" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B183" s="87" t="s">
+      <c r="B183" s="85" t="s">
         <v>1591</v>
       </c>
       <c r="C183" s="3" t="s">
@@ -15240,11 +15246,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="184" spans="1:18" ht="40.5">
+    <row r="184" spans="1:18" ht="40.5" hidden="1">
       <c r="A184" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B184" s="87" t="s">
+      <c r="B184" s="85" t="s">
         <v>1592</v>
       </c>
       <c r="C184" s="3" t="s">
@@ -15290,11 +15296,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="185" spans="1:18" ht="27">
+    <row r="185" spans="1:18" ht="27" hidden="1">
       <c r="A185" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B185" s="87" t="s">
+      <c r="B185" s="85" t="s">
         <v>1593</v>
       </c>
       <c r="C185" s="3" t="s">
@@ -15344,7 +15350,7 @@
       <c r="A186" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B186" s="87" t="s">
+      <c r="B186" s="85" t="s">
         <v>1594</v>
       </c>
       <c r="C186" s="3" t="s">
@@ -15386,11 +15392,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="187" spans="1:18" ht="27">
+    <row r="187" spans="1:18" ht="27" hidden="1">
       <c r="A187" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B187" s="87" t="s">
+      <c r="B187" s="85" t="s">
         <v>1595</v>
       </c>
       <c r="C187" s="3" t="s">
@@ -15430,11 +15436,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="188" spans="1:18" ht="43.5">
+    <row r="188" spans="1:18" ht="43.5" hidden="1">
       <c r="A188" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B188" s="87" t="s">
+      <c r="B188" s="85" t="s">
         <v>1596</v>
       </c>
       <c r="C188" s="3" t="s">
@@ -15482,11 +15488,11 @@
         <v>1330</v>
       </c>
     </row>
-    <row r="189" spans="1:18" ht="27">
+    <row r="189" spans="1:18" ht="27" hidden="1">
       <c r="A189" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="B189" s="87" t="s">
+      <c r="B189" s="85" t="s">
         <v>1597</v>
       </c>
       <c r="C189" s="3" t="s">
@@ -15538,11 +15544,11 @@
         <v>1340</v>
       </c>
     </row>
-    <row r="190" spans="1:18">
+    <row r="190" spans="1:18" hidden="1">
       <c r="A190" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B190" s="87" t="s">
+      <c r="B190" s="85" t="s">
         <v>1598</v>
       </c>
       <c r="C190" s="3" t="s">
@@ -15588,11 +15594,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="191" spans="1:18" ht="27">
+    <row r="191" spans="1:18" ht="27" hidden="1">
       <c r="A191" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B191" s="87" t="s">
+      <c r="B191" s="85" t="s">
         <v>1599</v>
       </c>
       <c r="C191" s="3" t="s">
@@ -15640,11 +15646,11 @@
         <v>1373</v>
       </c>
     </row>
-    <row r="192" spans="1:18" ht="43.5">
+    <row r="192" spans="1:18" ht="43.5" hidden="1">
       <c r="A192" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B192" s="87" t="s">
+      <c r="B192" s="85" t="s">
         <v>1600</v>
       </c>
       <c r="C192" s="3" t="s">
@@ -15687,11 +15693,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="193" spans="1:18" ht="27">
+    <row r="193" spans="1:18" ht="27" hidden="1">
       <c r="A193" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B193" s="87" t="s">
+      <c r="B193" s="85" t="s">
         <v>1601</v>
       </c>
       <c r="C193" s="3" t="s">
@@ -15738,7 +15744,7 @@
       <c r="A194" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B194" s="87" t="s">
+      <c r="B194" s="85" t="s">
         <v>1602</v>
       </c>
       <c r="C194" s="8" t="s">
@@ -15784,11 +15790,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="195" spans="1:18" ht="54">
+    <row r="195" spans="1:18" ht="54" hidden="1">
       <c r="A195" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B195" s="87" t="s">
+      <c r="B195" s="85" t="s">
         <v>1603</v>
       </c>
       <c r="C195" s="3" t="s">
@@ -15831,11 +15837,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="196" spans="1:18" ht="40.5">
+    <row r="196" spans="1:18" ht="54" hidden="1">
       <c r="A196" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B196" s="87" t="s">
+      <c r="B196" s="85" t="s">
         <v>1604</v>
       </c>
       <c r="C196" s="3" t="s">
@@ -15883,11 +15889,11 @@
         <v>1327</v>
       </c>
     </row>
-    <row r="197" spans="1:18" ht="40.5">
+    <row r="197" spans="1:18" ht="40.5" hidden="1">
       <c r="A197" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B197" s="87" t="s">
+      <c r="B197" s="85" t="s">
         <v>1605</v>
       </c>
       <c r="C197" s="3" t="s">
@@ -15937,7 +15943,7 @@
       <c r="A198" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B198" s="87" t="s">
+      <c r="B198" s="85" t="s">
         <v>1606</v>
       </c>
       <c r="C198" s="3" t="s">
@@ -15983,7 +15989,7 @@
       <c r="A199" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B199" s="87" t="s">
+      <c r="B199" s="85" t="s">
         <v>1607</v>
       </c>
       <c r="C199" s="3" t="s">
@@ -16026,11 +16032,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="200" spans="1:18">
+    <row r="200" spans="1:18" hidden="1">
       <c r="A200" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B200" s="87" t="s">
+      <c r="B200" s="85" t="s">
         <v>1608</v>
       </c>
       <c r="C200" s="3" t="s">
@@ -16076,11 +16082,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="201" spans="1:18" ht="29">
+    <row r="201" spans="1:18" ht="29" hidden="1">
       <c r="A201" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B201" s="87" t="s">
+      <c r="B201" s="85" t="s">
         <v>1609</v>
       </c>
       <c r="C201" s="3" t="s">
@@ -16132,11 +16138,11 @@
         <v>1336</v>
       </c>
     </row>
-    <row r="202" spans="1:18" ht="29">
+    <row r="202" spans="1:18" ht="29" hidden="1">
       <c r="A202" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B202" s="87" t="s">
+      <c r="B202" s="85" t="s">
         <v>1610</v>
       </c>
       <c r="C202" s="3" t="s">
@@ -16182,11 +16188,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="203" spans="1:18">
+    <row r="203" spans="1:18" hidden="1">
       <c r="A203" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B203" s="87" t="s">
+      <c r="B203" s="85" t="s">
         <v>1611</v>
       </c>
       <c r="C203" s="3" t="s">
@@ -16235,11 +16241,11 @@
         <v>1358</v>
       </c>
     </row>
-    <row r="204" spans="1:18" ht="58">
+    <row r="204" spans="1:18" ht="58" hidden="1">
       <c r="A204" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B204" s="87" t="s">
+      <c r="B204" s="85" t="s">
         <v>1612</v>
       </c>
       <c r="C204" s="3" t="s">
@@ -16281,11 +16287,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="205" spans="1:18">
+    <row r="205" spans="1:18" hidden="1">
       <c r="A205" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="B205" s="87" t="s">
+      <c r="B205" s="85" t="s">
         <v>1613</v>
       </c>
       <c r="C205" s="3" t="s">
@@ -16328,11 +16334,11 @@
         <v>981</v>
       </c>
     </row>
-    <row r="206" spans="1:18" ht="27">
+    <row r="206" spans="1:18" ht="27" hidden="1">
       <c r="A206" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B206" s="87" t="s">
+      <c r="B206" s="85" t="s">
         <v>1614</v>
       </c>
       <c r="C206" s="3" t="s">
@@ -16376,7 +16382,7 @@
       <c r="A207" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B207" s="87" t="s">
+      <c r="B207" s="85" t="s">
         <v>1615</v>
       </c>
       <c r="C207" s="3" t="s">
@@ -16416,11 +16422,11 @@
         <v>989</v>
       </c>
     </row>
-    <row r="208" spans="1:18" ht="27">
+    <row r="208" spans="1:18" ht="27" hidden="1">
       <c r="A208" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B208" s="87" t="s">
+      <c r="B208" s="85" t="s">
         <v>1616</v>
       </c>
       <c r="C208" s="3" t="s">
@@ -16466,11 +16472,11 @@
         <v>1355</v>
       </c>
     </row>
-    <row r="209" spans="1:18">
+    <row r="209" spans="1:18" hidden="1">
       <c r="A209" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B209" s="87" t="s">
+      <c r="B209" s="85" t="s">
         <v>1617</v>
       </c>
       <c r="C209" s="3" t="s">
@@ -16517,7 +16523,7 @@
       <c r="A210" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B210" s="87" t="s">
+      <c r="B210" s="85" t="s">
         <v>1618</v>
       </c>
       <c r="C210" s="8" t="s">
@@ -16573,7 +16579,7 @@
       <c r="A211" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B211" s="87" t="s">
+      <c r="B211" s="85" t="s">
         <v>1619</v>
       </c>
       <c r="C211" s="3" t="s">
@@ -16619,11 +16625,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="212" spans="1:18" ht="27">
+    <row r="212" spans="1:18" ht="27" hidden="1">
       <c r="A212" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B212" s="87" t="s">
+      <c r="B212" s="85" t="s">
         <v>1620</v>
       </c>
       <c r="C212" s="3" t="s">
@@ -16671,11 +16677,11 @@
         <v>1350</v>
       </c>
     </row>
-    <row r="213" spans="1:18" ht="27">
+    <row r="213" spans="1:18" ht="27" hidden="1">
       <c r="A213" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B213" s="87" t="s">
+      <c r="B213" s="85" t="s">
         <v>1621</v>
       </c>
       <c r="C213" s="3" t="s">
@@ -16725,7 +16731,7 @@
       <c r="A214" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B214" s="87" t="s">
+      <c r="B214" s="85" t="s">
         <v>1622</v>
       </c>
       <c r="C214" s="3" t="s">
@@ -16768,11 +16774,11 @@
         <v>1020</v>
       </c>
     </row>
-    <row r="215" spans="1:18" ht="27">
+    <row r="215" spans="1:18" ht="27" hidden="1">
       <c r="A215" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B215" s="87" t="s">
+      <c r="B215" s="85" t="s">
         <v>1623</v>
       </c>
       <c r="C215" s="3" t="s">
@@ -16815,11 +16821,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="216" spans="1:18" ht="40.5">
+    <row r="216" spans="1:18" ht="40.5" hidden="1">
       <c r="A216" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B216" s="87" t="s">
+      <c r="B216" s="85" t="s">
         <v>1624</v>
       </c>
       <c r="C216" s="3" t="s">
@@ -16873,7 +16879,7 @@
       <c r="A217" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B217" s="87" t="s">
+      <c r="B217" s="85" t="s">
         <v>1625</v>
       </c>
       <c r="C217" s="3" t="s">
@@ -16916,11 +16922,11 @@
         <v>1034</v>
       </c>
     </row>
-    <row r="218" spans="1:18" ht="40.5">
+    <row r="218" spans="1:18" ht="40.5" hidden="1">
       <c r="A218" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B218" s="87" t="s">
+      <c r="B218" s="85" t="s">
         <v>1626</v>
       </c>
       <c r="C218" s="3" t="s">
@@ -16963,11 +16969,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="219" spans="1:18" ht="27">
+    <row r="219" spans="1:18" ht="27" hidden="1">
       <c r="A219" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B219" s="87" t="s">
+      <c r="B219" s="85" t="s">
         <v>1627</v>
       </c>
       <c r="C219" s="3" t="s">
@@ -17013,11 +17019,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="220" spans="1:18" ht="27">
+    <row r="220" spans="1:18" ht="27" hidden="1">
       <c r="A220" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B220" s="87" t="s">
+      <c r="B220" s="85" t="s">
         <v>1628</v>
       </c>
       <c r="C220" s="3" t="s">
@@ -17069,11 +17075,11 @@
         <v>1346</v>
       </c>
     </row>
-    <row r="221" spans="1:18" ht="40.5">
+    <row r="221" spans="1:18" ht="40.5" hidden="1">
       <c r="A221" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B221" s="87" t="s">
+      <c r="B221" s="85" t="s">
         <v>1629</v>
       </c>
       <c r="C221" s="3" t="s">
@@ -17129,7 +17135,7 @@
       <c r="A222" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B222" s="87" t="s">
+      <c r="B222" s="85" t="s">
         <v>1630</v>
       </c>
       <c r="C222" s="3" t="s">
@@ -17175,11 +17181,11 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="223" spans="1:18" ht="27">
+    <row r="223" spans="1:18" ht="27" hidden="1">
       <c r="A223" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B223" s="87" t="s">
+      <c r="B223" s="85" t="s">
         <v>1631</v>
       </c>
       <c r="C223" s="3" t="s">
@@ -17229,7 +17235,7 @@
       <c r="A224" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B224" s="87" t="s">
+      <c r="B224" s="85" t="s">
         <v>1632</v>
       </c>
       <c r="C224" s="3" t="s">
@@ -17278,11 +17284,11 @@
         <v>1372</v>
       </c>
     </row>
-    <row r="225" spans="1:18" ht="29">
+    <row r="225" spans="1:18" ht="29" hidden="1">
       <c r="A225" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B225" s="87" t="s">
+      <c r="B225" s="85" t="s">
         <v>1633</v>
       </c>
       <c r="C225" s="3" t="s">
@@ -17318,11 +17324,11 @@
         <v>1072</v>
       </c>
     </row>
-    <row r="226" spans="1:18" ht="40.5">
+    <row r="226" spans="1:18" ht="40.5" hidden="1">
       <c r="A226" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B226" s="87" t="s">
+      <c r="B226" s="85" t="s">
         <v>1634</v>
       </c>
       <c r="C226" s="3" t="s">
@@ -17372,7 +17378,7 @@
       <c r="A227" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B227" s="87" t="s">
+      <c r="B227" s="85" t="s">
         <v>1635</v>
       </c>
       <c r="C227" s="3" t="s">
@@ -17412,11 +17418,11 @@
         <v>1359</v>
       </c>
     </row>
-    <row r="228" spans="1:18" ht="27">
+    <row r="228" spans="1:18" ht="27" hidden="1">
       <c r="A228" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B228" s="87" t="s">
+      <c r="B228" s="85" t="s">
         <v>1636</v>
       </c>
       <c r="C228" s="3" t="s">
@@ -17465,11 +17471,11 @@
         <v>1342</v>
       </c>
     </row>
-    <row r="229" spans="1:18" ht="40.5">
+    <row r="229" spans="1:18" ht="40.5" hidden="1">
       <c r="A229" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B229" s="87" t="s">
+      <c r="B229" s="85" t="s">
         <v>1637</v>
       </c>
       <c r="C229" s="3" t="s">
@@ -21141,11 +21147,11 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="29"/>
-      <c r="B1" s="85" t="s">
+      <c r="B1" s="87" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="85"/>
-      <c r="D1" s="85"/>
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="16"/>
@@ -21221,9 +21227,9 @@
       <c r="A10" s="28" t="s">
         <v>1211</v>
       </c>
-      <c r="B10" s="84"/>
-      <c r="C10" s="84"/>
-      <c r="D10" s="84"/>
+      <c r="B10" s="86"/>
+      <c r="C10" s="86"/>
+      <c r="D10" s="86"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -22868,12 +22874,9 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -23100,15 +23103,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE614213-7E3D-4CA8-9D43-54C11470A607}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{354A43F7-C600-406D-BA86-DE6617C712F8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="2fa8eba2-c100-4e42-af87-8a78c51844e9"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9fb94f25-3828-4f7c-9ced-948a50f90623"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -23133,18 +23148,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{354A43F7-C600-406D-BA86-DE6617C712F8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE614213-7E3D-4CA8-9D43-54C11470A607}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="2fa8eba2-c100-4e42-af87-8a78c51844e9"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9fb94f25-3828-4f7c-9ced-948a50f90623"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>